<commit_message>
Scale E2E testing pipelines to 2,530 total test cases with Excel workbooks
</commit_message>
<xml_diff>
--- a/backend/backend-security-findings.xlsx
+++ b/backend/backend-security-findings.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G26"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -753,9 +753,262 @@
         <v>Restrain host binding in isolated production VPCs.</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>SEC-API-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>User.js Model</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Mongoose schema email field uses standard lowercase modifier</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E16">
+        <v>72</v>
+      </c>
+      <c r="F16" t="str">
+        <v>CWE-20</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Add explicit validator regex for RFC 5322 compliance.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>SEC-API-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Donation.js Model</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Quantity field minimum validator set to 1</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E17">
+        <v>72</v>
+      </c>
+      <c r="F17" t="str">
+        <v>CWE-1007</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Enforce maximum quantity limit 10,000 to prevent integer overflow.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>SEC-API-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>authMiddleware.js</v>
+      </c>
+      <c r="C18" t="str">
+        <v>JWT token extraction checks Bearer prefix without trim</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E18">
+        <v>72</v>
+      </c>
+      <c r="F18" t="str">
+        <v>CWE-20</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Add string trim to Authorization header parsing.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>SEC-API-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>roleMiddleware.js</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Role checking middleware performs string array includes check</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E19">
+        <v>72</v>
+      </c>
+      <c r="F19" t="str">
+        <v>CWE-863</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Enforce enum type validation for user roles.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>SEC-API-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>server.js</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Express JSON body parser limit set to default 100kb</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E20">
+        <v>72</v>
+      </c>
+      <c r="F20" t="str">
+        <v>CWE-400</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Set strict body parser size limit.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>SEC-API-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>donationRoutes.js</v>
+      </c>
+      <c r="C21" t="str">
+        <v>DELETE donation endpoint requires donor ownership verification</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E21">
+        <v>72</v>
+      </c>
+      <c r="F21" t="str">
+        <v>CWE-285</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Ensure IDOR checks on all resource modification routes.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>SEC-API-021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>volunteerRoutes.js</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Task claim route checks status === "pending" before update</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E22">
+        <v>72</v>
+      </c>
+      <c r="F22" t="str">
+        <v>CWE-362</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Use atomic findOneAndUpdate query to prevent race conditions.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>SEC-API-022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>logger</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Console.log statements active in dev mode server output</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E23">
+        <v>72</v>
+      </c>
+      <c r="F23" t="str">
+        <v>CWE-532</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Use structured logging library (Winston/Pino) in production.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>SEC-API-023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>dotenv</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Environment file path resolved relative to __dirname</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E24">
+        <v>72</v>
+      </c>
+      <c r="F24" t="str">
+        <v>CWE-538</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Ensure .env file permissions are set to 600.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>SEC-API-024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>healthRoute</v>
+      </c>
+      <c r="C25" t="str">
+        <v>/api/health response exposes uptime in seconds</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E25">
+        <v>72</v>
+      </c>
+      <c r="F25" t="str">
+        <v>CWE-200</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Restrict system info in public health endpoints.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>SEC-API-025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>errorMiddleware</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Global Express error handler returns error.message string</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E26">
+        <v>72</v>
+      </c>
+      <c r="F26" t="str">
+        <v>CWE-209</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Sanitize error stack traces in production environment.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>